<commit_message>
Edit GMHO_Upper_Defs.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/UpperLevel/GMHO_Upper_Defs.xlsx
+++ b/UpperLevel/GMHO_Upper_Defs.xlsx
@@ -44,12 +44,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
+        <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002f4f4f"/>
+        <fgColor rgb="00ffffff"/>
       </patternFill>
     </fill>
   </fills>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA44"/>
+  <dimension ref="A1:AA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,122 +457,122 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>BFO entity</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has process part'</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has process attribute'</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'realises'</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has intervention outcome'</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'participates in'</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'investigates'</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has context'</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Curator note</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Definition source</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Cross reference</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Informal label for repository</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has part'</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>Informal definition</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>BFO entity</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has process part'</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has process attribute'</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'realises'</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has intervention outcome'</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'participates in'</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'investigates'</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has context'</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Definition source</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Cross reference</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Informal label for repository</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has part'</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Curator note</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>To be reviewed by</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
           <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>communication process attribute</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -619,12 +619,12 @@
           <t xml:space="preserve">A process context in which the process is an experience. </t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
@@ -648,12 +648,12 @@
       <c r="U3" s="2" t="n"/>
       <c r="V3" s="2" t="n"/>
       <c r="W3" s="2" t="n"/>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="X3" s="2" t="n"/>
+      <c r="Y3" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="n"/>
       <c r="Z3" s="2" t="n"/>
       <c r="AA3" s="2" t="n"/>
     </row>
@@ -673,12 +673,12 @@
           <t>An object aggregate consisting of an organism and all material entities located within the organism, overlapping the organism, or occupying sites formed in part by the organism.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -700,12 +700,12 @@
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -727,14 +727,19 @@
           <t>An object aggregate that consists of two or more people.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>target population</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>target population</t>
+          <t>This entity represents any group consisting of two or more people. It could range for example from small groups, neighbourhoods, and organisations to entire national populations.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -742,17 +747,12 @@
           <t>population history</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>This entity represents any group consisting of two or more people. It could range for example from small groups, neighbourhoods, and organisations to entire national populations.</t>
-        </is>
-      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -774,12 +774,12 @@
           <t>A process that is produced by a person.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -801,305 +801,297 @@
           <t>A planned process that has the aim of influencing an outcome.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000003</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>A process attribute whose bearer is an intervention.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="n"/>
-      <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
+      <c r="N9" s="3" t="n"/>
+      <c r="O9" s="3" t="n"/>
+      <c r="P9" s="3" t="n"/>
+      <c r="Q9" s="3" t="n"/>
+      <c r="R9" s="3" t="n"/>
+      <c r="S9" s="3" t="inlineStr">
         <is>
           <t>BCIO:050315</t>
         </is>
       </c>
-      <c r="T9" s="2" t="n"/>
-      <c r="U9" s="2" t="n"/>
-      <c r="V9" s="2" t="n"/>
-      <c r="W9" s="2" t="n"/>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Y9" s="2" t="n"/>
-      <c r="Z9" s="2" t="n"/>
-      <c r="AA9" s="2" t="n"/>
+      <c r="T9" s="3" t="n"/>
+      <c r="U9" s="3" t="n"/>
+      <c r="V9" s="3" t="n"/>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="3" t="n"/>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="n"/>
+      <c r="AA9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>BCIO:051010</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>BCIO:046000</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>intervention content</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000253</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention context
 </t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>A process context in which the process is an intervention.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="n"/>
-      <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="n"/>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="n"/>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">BCIO:005000
 </t>
         </is>
       </c>
-      <c r="T11" s="2" t="n"/>
-      <c r="U11" s="2" t="n"/>
-      <c r="V11" s="2" t="inlineStr">
+      <c r="T12" s="2" t="n"/>
+      <c r="U12" s="2" t="n"/>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>intervention setting; intervention temporal context; intervention population</t>
         </is>
       </c>
-      <c r="W11" s="2" t="n"/>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="W12" s="2" t="n"/>
+      <c r="X12" s="2" t="n"/>
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y11" s="2" t="n"/>
-      <c r="Z11" s="2" t="n"/>
-      <c r="AA11" s="2" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="Z12" s="2" t="n"/>
+      <c r="AA12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>BCIO:045000</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>intervention delivery</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>A planned process by which intervention content is delivered.</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>The planned process for delivering an intervention to its participants.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery; intervention style of delivery; intervention mode of delivery; intervention source</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>This class intends to represent the actual delivery of an intervention, whereas the class "mental health intervention scenario plan" refers to the planned intervention, including the planned delivery of an intervention. Distinguishing between these two classes allows for the assessment of intervention fidelity. To capture planned delivery, researchers could annotate both the class "intervention delivery" and "mental health intervention scenario plan".
 The definition of "intervention delivery" states that it is "a planned process by which intervention content is delivered," which refers to the actual execution of the intervention. This phrasing reflects that the intervention was designed and planned in advance before being implemented, thereby making it a "planned process".</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery; intervention style of delivery; intervention mode of delivery; intervention source</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>The planned process for delivering an intervention to its participants.</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000242</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention dose
 </t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>An intervention attribute that is its amount.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">drug dose and number of intervention techniques (e.g., action plans, social support)
 </t>
         </is>
       </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Intervention dose can capture the intensity of any intervention, including social, physical, psychological and pharmacological interventions.
 Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the classes "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose. This class intends to represent the actual dose delivered as part of an intervention, whereas the class "mental health intervention scenario plan" refers to the planned intervention, including the planned dose of an intervention. Distinguishing between these two classes allows for the assessment of intervention fidelity. To capture planned dose, researchers could annotate both the class "intervention dose" and "mental health intervention scenario plan".
 </t>
         </is>
       </c>
-      <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="n"/>
-      <c r="T13" s="2" t="n"/>
-      <c r="U13" s="2" t="n"/>
-      <c r="V13" s="2" t="n"/>
-      <c r="W13" s="2" t="n"/>
-      <c r="X13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Y13" s="2" t="n"/>
-      <c r="Z13" s="2" t="n"/>
-      <c r="AA13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000199</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>intervention mechanism of action</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>A process that is causally active in the relationship between an intervention scenario and its intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">For a construct to be a mechanism of action, it must be causally active in bringing about the intervention’s effect on its outcome. However, interventions are typically designed based on hypothesised mechanisms of action, which may or may not hold true depending on factors such as population and setting. 
-The ontology provides a structured framework for organising mechanisms of action but does not replace the need for empirical validation. The ontology does not specify the level of evidence required to confirm that a hypothesised mechanism has been realised. In other words, the ontology itself does not make causal inferences about specific mechanisms. 
-When using the ontology, researchers can code hypothesised mechanisms within the subclasses of “intervention mechanism of action”. The assessment of whether sufficient evidence supports a causal relationship occurs at the annotation level, where empirical data validate the connections between constructs. 
-The relationship between intervention techniques, mechanisms, and outcomes is often complex and non-linear. Multiple mechanisms of action may interact in various ways, including combinations, sequences, or feedback loops.
-</t>
-        </is>
-      </c>
+      <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
       <c r="Q14" s="2" t="n"/>
       <c r="R14" s="2" t="n"/>
@@ -1108,43 +1100,49 @@
       <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="n"/>
       <c r="W14" s="2" t="n"/>
-      <c r="X14" s="2" t="inlineStr">
+      <c r="X14" s="2" t="n"/>
+      <c r="Y14" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y14" s="2" t="n"/>
       <c r="Z14" s="2" t="n"/>
       <c r="AA14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000244</t>
+          <t>GMHO:0000199</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">intervention mode of delivery
-</t>
+          <t>intervention mechanism of action</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An intervention attribute that is the physical or informational medium through which an intervention is provided.
-</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
+          <t>A process that is causally active in the relationship between an intervention scenario and its intervention outcome.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For a construct to be a mechanism of action, it must be causally active in bringing about the intervention’s effect on its outcome. However, interventions are typically designed based on hypothesised mechanisms of action, which may or may not hold true depending on factors such as population and setting. 
+The ontology provides a structured framework for organising mechanisms of action but does not replace the need for empirical validation. The ontology does not specify the level of evidence required to confirm that a hypothesised mechanism has been realised. In other words, the ontology itself does not make causal inferences about specific mechanisms. 
+When using the ontology, researchers can code hypothesised mechanisms within the subclasses of “intervention mechanism of action”. The assessment of whether sufficient evidence supports a causal relationship occurs at the annotation level, where empirical data validate the connections between constructs. 
+The relationship between intervention techniques, mechanisms, and outcomes is often complex and non-linear. Multiple mechanisms of action may interact in various ways, including combinations, sequences, or feedback loops.
+</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
@@ -1159,152 +1157,152 @@
       <c r="U15" s="2" t="n"/>
       <c r="V15" s="2" t="n"/>
       <c r="W15" s="2" t="n"/>
-      <c r="X15" s="2" t="inlineStr">
+      <c r="X15" s="2" t="n"/>
+      <c r="Y15" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y15" s="2" t="n"/>
       <c r="Z15" s="2" t="n"/>
       <c r="AA15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>BCIO:039000</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>intervention outcome</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>An entity that is influenced by an intervention.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000244</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention mode of delivery
+</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An intervention attribute that is the physical or informational medium through which an intervention is provided.
+</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="n"/>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n"/>
+      <c r="V16" s="2" t="n"/>
+      <c r="W16" s="2" t="n"/>
+      <c r="X16" s="2" t="n"/>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="n"/>
+      <c r="AA16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>BCIO:039000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>intervention outcome</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>An entity that is influenced by an intervention.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>BCIO:015095</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>intervention population</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>The definition of intervention population (A human population who are exposed to an intervention) does not imply an explicit assignment to an intervention arm. While some interventions will have study designs in which researchers explicitly assign participants to intervention and control groups, this is not the case for all interventions (e.g., policy changes or public health campaigns).</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>mental health intervention scenario</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>The definition of intervention population (A human population who are exposed to an intervention) does not imply an explicit assignment to an intervention arm. While some interventions will have study designs in which researchers explicitly assign participants to intervention and control groups, this is not the case for all interventions (e.g., policy changes or public health campaigns).</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:009000</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>intervention schedule of delivery</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>An intervention attribute that is its temporal organisation.</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-      <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="3" t="inlineStr"/>
-      <c r="Q18" s="3" t="inlineStr"/>
-      <c r="R18" s="3" t="inlineStr"/>
-      <c r="S18" s="3" t="inlineStr"/>
-      <c r="T18" s="3" t="inlineStr"/>
-      <c r="U18" s="3" t="inlineStr"/>
-      <c r="V18" s="3" t="inlineStr"/>
-      <c r="W18" s="3" t="inlineStr"/>
-      <c r="X18" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="Y18" s="3" t="inlineStr"/>
-      <c r="Z18" s="3" t="inlineStr"/>
-      <c r="AA18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>GMHO:0000245</t>
+          <t>BCIO:009000</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">intervention schedule of delivery
-</t>
+          <t>intervention schedule of delivery</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">An intervention attribute that involves its temporal organisation.
-</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="inlineStr">
+          <t>An intervention attribute that is its temporal organisation.</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
+      <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
@@ -1314,13 +1312,7 @@
       <c r="L19" s="4" t="n"/>
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Temporal organisation includes different temporal dimensions, such as timing, frequency, duration and the sequence of activities.
-Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose.
-</t>
-        </is>
-      </c>
+      <c r="O19" s="4" t="n"/>
       <c r="P19" s="4" t="n"/>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
@@ -1329,101 +1321,97 @@
       <c r="U19" s="4" t="n"/>
       <c r="V19" s="4" t="n"/>
       <c r="W19" s="4" t="n"/>
-      <c r="X19" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="Y19" s="4" t="n"/>
+      <c r="X19" s="4" t="n"/>
+      <c r="Y19" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="Z19" s="4" t="n"/>
       <c r="AA19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000245</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention schedule of delivery
+</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An intervention attribute that involves its temporal organisation.
+</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporal organisation includes different temporal dimensions, such as timing, frequency, duration and the sequence of activities.
+Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose.
+</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="n"/>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="n"/>
+      <c r="R20" s="3" t="n"/>
+      <c r="S20" s="3" t="n"/>
+      <c r="T20" s="3" t="n"/>
+      <c r="U20" s="3" t="n"/>
+      <c r="V20" s="3" t="n"/>
+      <c r="W20" s="3" t="n"/>
+      <c r="X20" s="3" t="n"/>
+      <c r="Y20" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z20" s="3" t="n"/>
+      <c r="AA20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000169</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention setting
 </t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>An aggregate of entities that form the environment in which an intervention is provided.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCIO:005000
-</t>
-        </is>
-      </c>
-      <c r="T20" s="2" t="n"/>
-      <c r="U20" s="2" t="n"/>
-      <c r="V20" s="2" t="n"/>
-      <c r="W20" s="2" t="n"/>
-      <c r="X20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Y20" s="2" t="n"/>
-      <c r="Z20" s="2" t="n"/>
-      <c r="AA20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000246</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">intervention source
-</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A role played by a person, population or organisation that provides an intervention.
-</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">intervention provider
-</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
@@ -1431,51 +1419,112 @@
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The class “intervention source” has been defined to include a person, population or organisation, as these sources can be legally accountable for an intervention. A computer program or machine cannot be held accountable in the same way. Therefore, the organisation or people that provide the computer program or machine would be considered the intervention source, where relevant. When an intervention is delivered via a computer program (e.g., an app), this can be captured in the ontology through the relevant subclasses of "intervention mode of delivery".
-</t>
-        </is>
-      </c>
+      <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
       <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="n"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCIO:005000
+</t>
+        </is>
+      </c>
       <c r="T21" s="2" t="n"/>
       <c r="U21" s="2" t="n"/>
       <c r="V21" s="2" t="n"/>
       <c r="W21" s="2" t="n"/>
-      <c r="X21" s="2" t="inlineStr">
+      <c r="X21" s="2" t="n"/>
+      <c r="Y21" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y21" s="2" t="n"/>
       <c r="Z21" s="2" t="n"/>
       <c r="AA21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000246</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention source
+</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A role played by a person, population or organisation that provides an intervention.
+</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention provider
+</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The class “intervention source” has been defined to include a person, population or organisation, as these sources can be legally accountable for an intervention. A computer program or machine cannot be held accountable in the same way. Therefore, the organisation or people that provide the computer program or machine would be considered the intervention source, where relevant. When an intervention is delivered via a computer program (e.g., an app), this can be captured in the ontology through the relevant subclasses of "intervention mode of delivery".
+</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="2" t="n"/>
+      <c r="R22" s="2" t="n"/>
+      <c r="S22" s="2" t="n"/>
+      <c r="T22" s="2" t="n"/>
+      <c r="U22" s="2" t="n"/>
+      <c r="V22" s="2" t="n"/>
+      <c r="W22" s="2" t="n"/>
+      <c r="X22" s="2" t="n"/>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="n"/>
+      <c r="AA22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>BCIO:044005</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>intervention style of delivery</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>A communication style that is an attribute of an intervention content communication process.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>communication style</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>An intervention can include various different styles of delivery for different parts of the intervention.
 The definition of "intervention style of delivery" is based on two other entities, namely "communication style" and "intervention content communication process". Their definitions are presented below.
@@ -1483,83 +1532,34 @@
 intervention content communication process (BCIO:044001): A communication that transmits the content of an intervention Note that an intervention is a planned process with the aim of influencing some outcome whereas a behaviour change intervention is an intervention that aims to influence human behaviour as an outcome.</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000247</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>intervention technique</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that is the smallest part of an intervention that is observable, replicable and on its own has the potential to influence an intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="n"/>
-      <c r="X23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Y23" s="2" t="n"/>
-      <c r="Z23" s="2" t="n"/>
-      <c r="AA23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000254</t>
+          <t>GMHO:0000247</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal context</t>
+          <t>intervention technique</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">temporal context of process </t>
-        </is>
-      </c>
+          <t>A planned process that is the smallest part of an intervention that is observable, replicable and on its own has the potential to influence an intervention outcome.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
@@ -1573,47 +1573,42 @@
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="n"/>
       <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCIO:047000
-</t>
-        </is>
-      </c>
+      <c r="S24" s="2" t="n"/>
       <c r="T24" s="2" t="n"/>
       <c r="U24" s="2" t="n"/>
       <c r="V24" s="2" t="n"/>
       <c r="W24" s="2" t="n"/>
-      <c r="X24" s="2" t="inlineStr">
+      <c r="X24" s="2" t="n"/>
+      <c r="Y24" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y24" s="2" t="n"/>
       <c r="Z24" s="2" t="n"/>
       <c r="AA24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000004</t>
+          <t>GMHO:0000254</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>material context of process</t>
+          <t>intervention temporal context</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A material entity that is not dependent on a process but may influence the effect of the process on its outcome. </t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temporal context of process </t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
@@ -1627,66 +1622,57 @@
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="n"/>
       <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="n"/>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCIO:047000
+</t>
+        </is>
+      </c>
       <c r="T25" s="2" t="n"/>
       <c r="U25" s="2" t="n"/>
       <c r="V25" s="2" t="n"/>
       <c r="W25" s="2" t="n"/>
-      <c r="X25" s="2" t="inlineStr">
+      <c r="X25" s="2" t="n"/>
+      <c r="Y25" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y25" s="2" t="n"/>
       <c r="Z25" s="2" t="n"/>
       <c r="AA25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000248</t>
+          <t>GMHO:0000004</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mental health intervention
-</t>
+          <t>material context of process</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>An intervention that has the aim of influencing some aspect of mental health.</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
+          <t xml:space="preserve">A material entity that is not dependent on a process but may influence the effect of the process on its outcome. </t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>intervention delivery; mental health intervention content</t>
-        </is>
-      </c>
+      <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
+      <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context, level of engagement and outcomes. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. 
-</t>
-        </is>
-      </c>
+      <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
@@ -1695,58 +1681,59 @@
       <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="n"/>
       <c r="W26" s="2" t="n"/>
-      <c r="X26" s="2" t="inlineStr">
+      <c r="X26" s="2" t="n"/>
+      <c r="Y26" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y26" s="2" t="n"/>
       <c r="Z26" s="2" t="n"/>
       <c r="AA26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000241</t>
+          <t>GMHO:0000248</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mental health intervention content
+          <t xml:space="preserve">mental health intervention
 </t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>An intervention content that is part of a mental health intervention.</t>
+          <t>An intervention that has the aim of influencing some aspect of mental health.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Any intervention content delivered in the context of a mental health intervention.</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>intervention content</t>
-        </is>
-      </c>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context, level of engagement and outcomes. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. 
+</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>intervention technique</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>intervention dose</t>
-        </is>
-      </c>
+          <t>intervention delivery; mental health intervention content</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="n"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>participant engagement with intervention</t>
+        </is>
+      </c>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
@@ -1757,209 +1744,229 @@
       <c r="U27" s="2" t="n"/>
       <c r="V27" s="2" t="n"/>
       <c r="W27" s="2" t="n"/>
-      <c r="X27" s="2" t="inlineStr">
+      <c r="X27" s="2" t="n"/>
+      <c r="Y27" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y27" s="2" t="n"/>
       <c r="Z27" s="2" t="n"/>
       <c r="AA27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000250</t>
+          <t>GMHO:0000241</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario</t>
+          <t xml:space="preserve">mental health intervention content
+</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>A planned process in which a mental health intervention is applied in a given context.</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
+          <t>An intervention content that is part of a mental health intervention.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>intervention mechanism of action; participant engagement with intervention; mental health intervention</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention scenario plan</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>intervention outcome</t>
-        </is>
-      </c>
+          <t>intervention technique</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>intervention dose</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n"/>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. </t>
-        </is>
-      </c>
+      <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="n"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>intervention context</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="n"/>
       <c r="R28" s="2" t="n"/>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="2" t="n"/>
-      <c r="U28" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
+      <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="n"/>
       <c r="W28" s="2" t="n"/>
       <c r="X28" s="2" t="inlineStr">
         <is>
+          <t>Any intervention content delivered in the context of a mental health intervention.</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y28" s="2" t="n"/>
       <c r="Z28" s="2" t="n"/>
       <c r="AA28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000260</t>
+          <t>GMHO:0000250</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario plan</t>
+          <t>mental health intervention scenario</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A plan that is realized in a mental health intervention scenario process.</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>plan</t>
-        </is>
-      </c>
+          <t>A planned process in which a mental health intervention is applied in a given context.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
-      <c r="J29" s="2" t="n"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. </t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>intervention mechanism of action; participant engagement with intervention; mental health intervention</t>
+        </is>
+      </c>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="n"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>intervention outcome</t>
+        </is>
+      </c>
       <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>This class is intended to represent the planned content or delivery of an intervention, whereas the class "mental health intervention scenario" refers to the intervention as it was actually implemented. Distinguishing between these two classes allows for the assessment of intervention fidelity.</t>
-        </is>
-      </c>
+      <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="n"/>
-      <c r="Q29" s="2" t="n"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
       <c r="R29" s="2" t="n"/>
-      <c r="S29" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:028000</t>
-        </is>
-      </c>
+      <c r="S29" s="2" t="n"/>
       <c r="T29" s="2" t="n"/>
-      <c r="U29" s="2" t="n"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
       <c r="V29" s="2" t="n"/>
       <c r="W29" s="2" t="n"/>
-      <c r="X29" s="2" t="inlineStr">
+      <c r="X29" s="2" t="n"/>
+      <c r="Y29" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y29" s="2" t="n"/>
       <c r="Z29" s="2" t="n"/>
       <c r="AA29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>BFO:0000027</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">b is an object aggregate means: b is a material entity consisting exactly of a plurality of objects as member_parts at all times at which b exists. </t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000260</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>A plan that is realized in a mental health intervention scenario process.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>This class is intended to represent the planned content or delivery of an intervention, whereas the class "mental health intervention scenario" refers to the intervention as it was actually implemented. Distinguishing between these two classes allows for the assessment of intervention fidelity.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2" t="n"/>
+      <c r="O30" s="2" t="n"/>
+      <c r="P30" s="2" t="n"/>
+      <c r="Q30" s="2" t="n"/>
+      <c r="R30" s="2" t="n"/>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:028000</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="n"/>
+      <c r="U30" s="2" t="n"/>
+      <c r="V30" s="2" t="n"/>
+      <c r="W30" s="2" t="n"/>
+      <c r="X30" s="2" t="n"/>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="n"/>
+      <c r="AA30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BCIO:050916</t>
+          <t>BFO:0000027</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>participant engagement with intervention</t>
+          <t>object aggregate</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
+          <t xml:space="preserve">b is an object aggregate means: b is a material entity consisting exactly of a plurality of objects as member_parts at all times at which b exists. </t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>The extent to which someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attendance to intervention sessions, participation in intervention activities, emotionally engaging with intervention content </t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Engagement can involve cognitive, emotional and behavioural engagement with an intervention.</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1968,30 +1975,40 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MF:0000016</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>person</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>An extended organism that is a member of the species Homo sapiens.</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>extended organism</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>personal history</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>individual human activity</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attendance to intervention sessions, participation in intervention activities, emotionally engaging with intervention content </t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Engagement can involve cognitive, emotional and behavioural engagement with an intervention.</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
+        <is>
+          <t>The extent to which someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -2000,40 +2017,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BCIO:015161</t>
+          <t>MF:0000016</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>An extended organism that is a member of the species Homo sapiens.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>extended organism</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
           <t>personal history</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>A history that is of a person.</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>history</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>sum of multiple experienced events</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>A person's history includes the sum of their experiences, which can include experiences relating to their cultural, social and economic context.</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
+      <c r="Y33" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -2042,35 +2049,40 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BCIO:050487</t>
+          <t>BCIO:015161</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>personal history</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>A history that is of a person.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>sum of multiple experienced events</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>A person's history includes the sum of their experiences, which can include experiences relating to their cultural, social and economic context.</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>A process that is part of a personal history.</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>experienced event</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>context of experience</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -2079,25 +2091,35 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OBI:0000260</t>
+          <t>BCIO:050487</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>personal history part</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+          <t>A process that is part of a personal history.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>process</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
+          <t>experienced event</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>context of experience</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -2106,167 +2128,141 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>OBI:0000260</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>OBI:0000011</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>A process that realizes a plan which is the concretization of a plan specification.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="Y37" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000251</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>population history</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>A history that is of a population.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>history</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
-      <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>is an aggregate of personal history; experiences can be captured as 'personal history part'.</t>
         </is>
       </c>
-      <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="n"/>
-      <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="n"/>
-      <c r="T37" s="2" t="n"/>
-      <c r="U37" s="2" t="n"/>
-      <c r="V37" s="2" t="n"/>
-      <c r="W37" s="2" t="n"/>
-      <c r="X37" s="2" t="inlineStr">
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
+      <c r="N38" s="2" t="n"/>
+      <c r="O38" s="2" t="n"/>
+      <c r="P38" s="2" t="n"/>
+      <c r="Q38" s="2" t="n"/>
+      <c r="R38" s="2" t="n"/>
+      <c r="S38" s="2" t="n"/>
+      <c r="T38" s="2" t="n"/>
+      <c r="U38" s="2" t="n"/>
+      <c r="V38" s="2" t="n"/>
+      <c r="W38" s="2" t="n"/>
+      <c r="X38" s="2" t="n"/>
+      <c r="Y38" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y37" s="2" t="n"/>
-      <c r="Z37" s="2" t="n"/>
-      <c r="AA37" s="2" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="Z38" s="2" t="n"/>
+      <c r="AA38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>BFO:0000015</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>p is a process = Def. p is an occurrent that has temporal proper parts and for some time t, p s-depends_on some material entity at t. (axiom label in BFO2 Reference: [083-003])</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
+      <c r="Y39" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>GMHO:0000005</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">'temporal context of process' OR 'material context of process' </t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="4" t="n"/>
-      <c r="J39" s="4" t="n"/>
-      <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="n"/>
-      <c r="M39" s="4" t="n"/>
-      <c r="N39" s="4" t="n"/>
-      <c r="O39" s="4" t="n"/>
-      <c r="P39" s="4" t="n"/>
-      <c r="Q39" s="4" t="n"/>
-      <c r="R39" s="4" t="n"/>
-      <c r="S39" s="4" t="n"/>
-      <c r="T39" s="4" t="n"/>
-      <c r="U39" s="4" t="n"/>
-      <c r="V39" s="4" t="n"/>
-      <c r="W39" s="4" t="n"/>
-      <c r="X39" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="Y39" s="4" t="n"/>
-      <c r="Z39" s="4" t="n"/>
-      <c r="AA39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>GMHO:0000268</t>
+          <t>GMHO:0000005</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2279,15 +2275,15 @@
           <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
+      <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>'temporal context of process' OR 'material context of process'</t>
+          <t xml:space="preserve">'temporal context of process' OR 'material context of process' </t>
         </is>
       </c>
       <c r="G40" s="3" t="n"/>
@@ -2307,179 +2303,232 @@
       <c r="U40" s="3" t="n"/>
       <c r="V40" s="3" t="n"/>
       <c r="W40" s="3" t="n"/>
-      <c r="X40" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="Y40" s="3" t="n"/>
+      <c r="X40" s="3" t="n"/>
+      <c r="Y40" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="Z40" s="3" t="n"/>
       <c r="AA40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>GMHO:0000268</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="n"/>
+      <c r="L41" s="4" t="n"/>
+      <c r="M41" s="4" t="n"/>
+      <c r="N41" s="4" t="n"/>
+      <c r="O41" s="4" t="n"/>
+      <c r="P41" s="4" t="n"/>
+      <c r="Q41" s="4" t="n"/>
+      <c r="R41" s="4" t="n"/>
+      <c r="S41" s="4" t="n"/>
+      <c r="T41" s="4" t="n"/>
+      <c r="U41" s="4" t="n"/>
+      <c r="V41" s="4" t="n"/>
+      <c r="W41" s="4" t="n"/>
+      <c r="X41" s="4" t="n"/>
+      <c r="Y41" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="Z41" s="4" t="n"/>
+      <c r="AA41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>SEPIO:0000125</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>research study</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="Y42" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000268</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>research study</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
         </is>
       </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
-      <c r="K42" s="4" t="n"/>
-      <c r="L42" s="4" t="n"/>
-      <c r="M42" s="4" t="n"/>
-      <c r="N42" s="4" t="n"/>
-      <c r="O42" s="4" t="n"/>
-      <c r="P42" s="4" t="n"/>
-      <c r="Q42" s="4" t="n"/>
-      <c r="R42" s="4" t="n"/>
-      <c r="S42" s="4" t="inlineStr">
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="3" t="n"/>
+      <c r="O43" s="3" t="n"/>
+      <c r="P43" s="3" t="n"/>
+      <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="3" t="n"/>
+      <c r="S43" s="3" t="inlineStr">
         <is>
           <t>SEPIO:0000125</t>
         </is>
       </c>
-      <c r="T42" s="4" t="n"/>
-      <c r="U42" s="4" t="n"/>
-      <c r="V42" s="4" t="n"/>
-      <c r="W42" s="4" t="n"/>
-      <c r="X42" s="4" t="inlineStr">
+      <c r="T43" s="3" t="n"/>
+      <c r="U43" s="3" t="n"/>
+      <c r="V43" s="3" t="n"/>
+      <c r="W43" s="3" t="n"/>
+      <c r="X43" s="3" t="n"/>
+      <c r="Y43" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="Y42" s="4" t="n"/>
-      <c r="Z42" s="4" t="n"/>
-      <c r="AA42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="Z43" s="3" t="n"/>
+      <c r="AA43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>BFO:0000023</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>A realizable entity the manifestation of which brings about some result or end that is not essential to a continuant in virtue of the kind of thing that it is but that can be served or participated in by that kind of continuant in some kinds of natural, social or institutional contexts.</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
+      <c r="Y44" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000006</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>temporal context of process</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">An occurrent that is not dependent on a process but may influence the effect of the process on its outcome. </t>
         </is>
       </c>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="n"/>
-      <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This entity includes time periods, events, etc. </t>
         </is>
       </c>
-      <c r="P44" s="2" t="n"/>
-      <c r="Q44" s="2" t="n"/>
-      <c r="R44" s="2" t="n"/>
-      <c r="S44" s="2" t="n"/>
-      <c r="T44" s="2" t="n"/>
-      <c r="U44" s="2" t="n"/>
-      <c r="V44" s="2" t="n"/>
-      <c r="W44" s="2" t="n"/>
-      <c r="X44" s="2" t="inlineStr">
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
+      <c r="M45" s="2" t="n"/>
+      <c r="N45" s="2" t="n"/>
+      <c r="O45" s="2" t="n"/>
+      <c r="P45" s="2" t="n"/>
+      <c r="Q45" s="2" t="n"/>
+      <c r="R45" s="2" t="n"/>
+      <c r="S45" s="2" t="n"/>
+      <c r="T45" s="2" t="n"/>
+      <c r="U45" s="2" t="n"/>
+      <c r="V45" s="2" t="n"/>
+      <c r="W45" s="2" t="n"/>
+      <c r="X45" s="2" t="n"/>
+      <c r="Y45" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="Y44" s="2" t="n"/>
-      <c r="Z44" s="2" t="n"/>
-      <c r="AA44" s="2" t="n"/>
+      <c r="Z45" s="2" t="n"/>
+      <c r="AA45" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update intervention schedule of delivery in GMHO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/UpperLevel/GMHO_Upper_Defs.xlsx
+++ b/UpperLevel/GMHO_Upper_Defs.xlsx
@@ -891,33 +891,11 @@
           <t>process attribute</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1282,53 +1260,37 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>BCIO:009000</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>An intervention attribute that is its temporal organisation.</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="4" t="n"/>
-      <c r="T19" s="4" t="n"/>
-      <c r="U19" s="4" t="n"/>
-      <c r="V19" s="4" t="n"/>
-      <c r="W19" s="4" t="n"/>
-      <c r="X19" s="4" t="n"/>
-      <c r="Y19" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="Z19" s="4" t="n"/>
-      <c r="AA19" s="4" t="n"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Temporal organisation includes different temporal dimensions, such as timing, frequency, duration and the sequence of activities.
+Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose.</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Edit GMHO_Upper_Defs.xlsx: update 4, add 4
</commit_message>
<xml_diff>
--- a/UpperLevel/GMHO_Upper_Defs.xlsx
+++ b/UpperLevel/GMHO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA45"/>
+  <dimension ref="A1:AA49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -925,199 +919,199 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BCIO:051025</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A process context in which the process is an intervention.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>intervention setting; intervention temporal context; intervention population</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000253</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention context
 </t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>A process context in which the process is an intervention.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="n"/>
-      <c r="R12" s="2" t="n"/>
-      <c r="S12" s="2" t="inlineStr">
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>This class has been replaced by the identical class BCIO:051025 in the Behaviour Change Intervention Ontology (BCIO). Use BCIO:051025 instead.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="n"/>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">BCIO:005000
 </t>
         </is>
       </c>
-      <c r="T12" s="2" t="n"/>
-      <c r="U12" s="2" t="n"/>
-      <c r="V12" s="2" t="inlineStr">
+      <c r="T13" s="3" t="n"/>
+      <c r="U13" s="3" t="n"/>
+      <c r="V13" s="3" t="inlineStr">
         <is>
           <t>intervention setting; intervention temporal context; intervention population</t>
         </is>
       </c>
-      <c r="W12" s="2" t="n"/>
-      <c r="X12" s="2" t="n"/>
-      <c r="Y12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z12" s="2" t="n"/>
-      <c r="AA12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="W13" s="3" t="n"/>
+      <c r="X13" s="3" t="n"/>
+      <c r="Y13" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z13" s="3" t="n"/>
+      <c r="AA13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>BCIO:045000</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>intervention delivery</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>A planned process by which intervention content is delivered.</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>This class intends to represent the actual delivery of an intervention, whereas the class "mental health intervention scenario plan" refers to the planned intervention, including the planned delivery of an intervention. Distinguishing between these two classes allows for the assessment of intervention fidelity. To capture planned delivery, researchers could annotate both the class "intervention delivery" and "mental health intervention scenario plan".
 The definition of "intervention delivery" states that it is "a planned process by which intervention content is delivered," which refers to the actual execution of the intervention. This phrasing reflects that the intervention was designed and planned in advance before being implemented, thereby making it a "planned process".</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>intervention schedule of delivery; intervention style of delivery; intervention mode of delivery; intervention source</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>The planned process for delivering an intervention to its participants.</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000242</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention dose
 </t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>An intervention attribute that is its amount.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">drug dose and number of intervention techniques (e.g., action plans, social support)
 </t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Intervention dose can capture the intensity of any intervention, including social, physical, psychological and pharmacological interventions.
 Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the classes "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose. This class intends to represent the actual dose delivered as part of an intervention, whereas the class "mental health intervention scenario plan" refers to the planned intervention, including the planned dose of an intervention. Distinguishing between these two classes allows for the assessment of intervention fidelity. To capture planned dose, researchers could annotate both the class "intervention dose" and "mental health intervention scenario plan".
-</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="n"/>
-      <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="n"/>
-      <c r="T14" s="2" t="n"/>
-      <c r="U14" s="2" t="n"/>
-      <c r="V14" s="2" t="n"/>
-      <c r="W14" s="2" t="n"/>
-      <c r="X14" s="2" t="n"/>
-      <c r="Y14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z14" s="2" t="n"/>
-      <c r="AA14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000199</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>intervention mechanism of action</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>A process that is causally active in the relationship between an intervention scenario and its intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">For a construct to be a mechanism of action, it must be causally active in bringing about the intervention’s effect on its outcome. However, interventions are typically designed based on hypothesised mechanisms of action, which may or may not hold true depending on factors such as population and setting. 
-The ontology provides a structured framework for organising mechanisms of action but does not replace the need for empirical validation. The ontology does not specify the level of evidence required to confirm that a hypothesised mechanism has been realised. In other words, the ontology itself does not make causal inferences about specific mechanisms. 
-When using the ontology, researchers can code hypothesised mechanisms within the subclasses of “intervention mechanism of action”. The assessment of whether sufficient evidence supports a causal relationship occurs at the annotation level, where empirical data validate the connections between constructs. 
-The relationship between intervention techniques, mechanisms, and outcomes is often complex and non-linear. Multiple mechanisms of action may interact in various ways, including combinations, sequences, or feedback loops.
 </t>
         </is>
       </c>
@@ -1147,31 +1141,37 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000244</t>
+          <t>GMHO:0000199</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">intervention mode of delivery
-</t>
+          <t>intervention mechanism of action</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An intervention attribute that is the physical or informational medium through which an intervention is provided.
-</t>
+          <t>A process that is causally active in the relationship between an intervention scenario and its intervention outcome.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>intervention attribute</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For a construct to be a mechanism of action, it must be causally active in bringing about the intervention’s effect on its outcome. However, interventions are typically designed based on hypothesised mechanisms of action, which may or may not hold true depending on factors such as population and setting. 
+The ontology provides a structured framework for organising mechanisms of action but does not replace the need for empirical validation. The ontology does not specify the level of evidence required to confirm that a hypothesised mechanism has been realised. In other words, the ontology itself does not make causal inferences about specific mechanisms. 
+When using the ontology, researchers can code hypothesised mechanisms within the subclasses of “intervention mechanism of action”. The assessment of whether sufficient evidence supports a causal relationship occurs at the annotation level, where empirical data validate the connections between constructs. 
+The relationship between intervention techniques, mechanisms, and outcomes is often complex and non-linear. Multiple mechanisms of action may interact in various ways, including combinations, sequences, or feedback loops.
+</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
@@ -1196,61 +1196,75 @@
       <c r="AA16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>BCIO:039000</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>intervention outcome</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>An entity that is influenced by an intervention.</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000244</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention mode of delivery
+</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An intervention attribute that is the physical or informational medium through which an intervention is provided.
+</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2" t="n"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="n"/>
+      <c r="R17" s="2" t="n"/>
+      <c r="S17" s="2" t="n"/>
+      <c r="T17" s="2" t="n"/>
+      <c r="U17" s="2" t="n"/>
+      <c r="V17" s="2" t="n"/>
+      <c r="W17" s="2" t="n"/>
+      <c r="X17" s="2" t="n"/>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="n"/>
+      <c r="AA17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BCIO:015095</t>
+          <t>BCIO:039000</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>intervention population</t>
+          <t>intervention outcome</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A human population who are exposed to an intervention.</t>
+          <t>An entity that is influenced by an intervention.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>human population</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>The definition of intervention population (A human population who are exposed to an intervention) does not imply an explicit assignment to an intervention arm. While some interventions will have study designs in which researchers explicitly assign participants to intervention and control groups, this is not the case for all interventions (e.g., policy changes or public health campaigns).</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>mental health intervention scenario</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -1262,186 +1276,157 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>BCIO:015095</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>intervention population</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A human population who are exposed to an intervention.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>The definition of intervention population (A human population who are exposed to an intervention) does not imply an explicit assignment to an intervention arm. While some interventions will have study designs in which researchers explicitly assign participants to intervention and control groups, this is not the case for all interventions (e.g., policy changes or public health campaigns).</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>BCIO:009000</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>intervention schedule of delivery</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>An intervention attribute that is its temporal organisation.</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Temporal organisation includes different temporal dimensions, such as timing, frequency, duration and the sequence of activities.
 Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose.</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000245</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention schedule of delivery
 </t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">An intervention attribute that involves its temporal organisation.
 </t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Temporal organisation includes different temporal dimensions, such as timing, frequency, duration and the sequence of activities.
 Intervention dose refers to the intensity or amount of an intervention, which is about the content of an intervention. In contrast, an intervention's schedule of delivery is about the temporal aspects of the intervention. There is some overlap between the entities "intervention dose" and "intervention schedule of delivery". For example, a more frequent intervention schedule with specific doses would suggest a higher overall dose of the intervention. However, "intervention dose" can capture concepts that are not directly relevant to the temporal organisation of the intervention, such as overall number of intervention strategies and drug dose.
 </t>
         </is>
       </c>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
-      <c r="P20" s="3" t="n"/>
-      <c r="Q20" s="3" t="n"/>
-      <c r="R20" s="3" t="n"/>
-      <c r="S20" s="3" t="n"/>
-      <c r="T20" s="3" t="n"/>
-      <c r="U20" s="3" t="n"/>
-      <c r="V20" s="3" t="n"/>
-      <c r="W20" s="3" t="n"/>
-      <c r="X20" s="3" t="n"/>
-      <c r="Y20" s="3" t="inlineStr">
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="n"/>
+      <c r="P21" s="3" t="n"/>
+      <c r="Q21" s="3" t="n"/>
+      <c r="R21" s="3" t="n"/>
+      <c r="S21" s="3" t="n"/>
+      <c r="T21" s="3" t="n"/>
+      <c r="U21" s="3" t="n"/>
+      <c r="V21" s="3" t="n"/>
+      <c r="W21" s="3" t="n"/>
+      <c r="X21" s="3" t="n"/>
+      <c r="Y21" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="Z20" s="3" t="n"/>
-      <c r="AA20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="Z21" s="3" t="n"/>
+      <c r="AA21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>GMHO:0000169</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">intervention setting
 </t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>An aggregate of entities that form the environment in which an intervention is provided.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCIO:005000
-</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n"/>
-      <c r="U21" s="2" t="n"/>
-      <c r="V21" s="2" t="n"/>
-      <c r="W21" s="2" t="n"/>
-      <c r="X21" s="2" t="n"/>
-      <c r="Y21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z21" s="2" t="n"/>
-      <c r="AA21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000246</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">intervention source
-</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A role played by a person, population or organisation that provides an intervention.
-</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">intervention provider
-</t>
-        </is>
-      </c>
+      <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The class “intervention source” has been defined to include a person, population or organisation, as these sources can be legally accountable for an intervention. A computer program or machine cannot be held accountable in the same way. Therefore, the organisation or people that provide the computer program or machine would be considered the intervention source, where relevant. When an intervention is delivered via a computer program (e.g., an app), this can be captured in the ontology through the relevant subclasses of "intervention mode of delivery".
-</t>
-        </is>
-      </c>
+      <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
@@ -1451,7 +1436,12 @@
       <c r="P22" s="2" t="n"/>
       <c r="Q22" s="2" t="n"/>
       <c r="R22" s="2" t="n"/>
-      <c r="S22" s="2" t="n"/>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCIO:005000
+</t>
+        </is>
+      </c>
       <c r="T22" s="2" t="n"/>
       <c r="U22" s="2" t="n"/>
       <c r="V22" s="2" t="n"/>
@@ -1466,27 +1456,88 @@
       <c r="AA22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000246</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention source
+</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A role played by a person, population or organisation that provides an intervention.
+</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">intervention provider
+</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The class “intervention source” has been defined to include a person, population or organisation, as these sources can be legally accountable for an intervention. A computer program or machine cannot be held accountable in the same way. Therefore, the organisation or people that provide the computer program or machine would be considered the intervention source, where relevant. When an intervention is delivered via a computer program (e.g., an app), this can be captured in the ontology through the relevant subclasses of "intervention mode of delivery".
+</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2" t="n"/>
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="n"/>
+      <c r="S23" s="2" t="n"/>
+      <c r="T23" s="2" t="n"/>
+      <c r="U23" s="2" t="n"/>
+      <c r="V23" s="2" t="n"/>
+      <c r="W23" s="2" t="n"/>
+      <c r="X23" s="2" t="n"/>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="n"/>
+      <c r="AA23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>BCIO:044005</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>intervention style of delivery</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>A communication style that is an attribute of an intervention content communication process.</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>communication style</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>An intervention can include various different styles of delivery for different parts of the intervention.
 The definition of "intervention style of delivery" is based on two other entities, namely "communication style" and "intervention content communication process". Their definitions are presented below.
@@ -1494,80 +1545,31 @@
 intervention content communication process (BCIO:044001): A communication that transmits the content of an intervention Note that an intervention is a planned process with the aim of influencing some outcome whereas a behaviour change intervention is an intervention that aims to influence human behaviour as an outcome.</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000247</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>intervention technique</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that is the smallest part of an intervention that is observable, replicable and on its own has the potential to influence an intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="n"/>
-      <c r="T24" s="2" t="n"/>
-      <c r="U24" s="2" t="n"/>
-      <c r="V24" s="2" t="n"/>
-      <c r="W24" s="2" t="n"/>
-      <c r="X24" s="2" t="n"/>
-      <c r="Y24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z24" s="2" t="n"/>
-      <c r="AA24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000254</t>
+          <t>GMHO:0000247</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal context</t>
+          <t>intervention technique</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
+          <t>A planned process that is the smallest part of an intervention that is observable, replicable and on its own has the potential to influence an intervention outcome.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">temporal context of process </t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
@@ -1584,12 +1586,7 @@
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="n"/>
       <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCIO:047000
-</t>
-        </is>
-      </c>
+      <c r="S25" s="2" t="n"/>
       <c r="T25" s="2" t="n"/>
       <c r="U25" s="2" t="n"/>
       <c r="V25" s="2" t="n"/>
@@ -1604,137 +1601,131 @@
       <c r="AA25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000004</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>material context of process</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A material entity that is not dependent on a process but may influence the effect of the process on its outcome. </t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="n"/>
-      <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="n"/>
-      <c r="T26" s="2" t="n"/>
-      <c r="U26" s="2" t="n"/>
-      <c r="V26" s="2" t="n"/>
-      <c r="W26" s="2" t="n"/>
-      <c r="X26" s="2" t="n"/>
-      <c r="Y26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z26" s="2" t="n"/>
-      <c r="AA26" s="2" t="n"/>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000254</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>intervention temporal context</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temporal context of process </t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>This class has been replaced by the identical class BCIO:051026 in the Behaviour Change Intervention Ontology (BCIO). Use BCIO:051026 instead.</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
+      <c r="O26" s="3" t="n"/>
+      <c r="P26" s="3" t="n"/>
+      <c r="Q26" s="3" t="n"/>
+      <c r="R26" s="3" t="n"/>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCIO:047000
+</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="n"/>
+      <c r="U26" s="3" t="n"/>
+      <c r="V26" s="3" t="n"/>
+      <c r="W26" s="3" t="n"/>
+      <c r="X26" s="3" t="n"/>
+      <c r="Y26" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z26" s="3" t="n"/>
+      <c r="AA26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000248</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mental health intervention
-</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>An intervention that has the aim of influencing some aspect of mental health.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context, level of engagement and outcomes. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. 
-</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>intervention delivery; mental health intervention content</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="n"/>
-      <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="n"/>
-      <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="n"/>
-      <c r="U27" s="2" t="n"/>
-      <c r="V27" s="2" t="n"/>
-      <c r="W27" s="2" t="n"/>
-      <c r="X27" s="2" t="n"/>
-      <c r="Y27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z27" s="2" t="n"/>
-      <c r="AA27" s="2" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BCIO:051026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>intervention temporal context</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000241</t>
+          <t>GMHO:0000004</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mental health intervention content
-</t>
+          <t>material context of process</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>An intervention content that is part of a mental health intervention.</t>
+          <t xml:space="preserve">A material entity that is not dependent on a process but may influence the effect of the process on its outcome. </t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>intervention content</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="E28" s="2" t="n"/>
@@ -1742,16 +1733,8 @@
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>intervention technique</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>intervention dose</t>
-        </is>
-      </c>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="n"/>
       <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n"/>
@@ -1764,11 +1747,7 @@
       <c r="U28" s="2" t="n"/>
       <c r="V28" s="2" t="n"/>
       <c r="W28" s="2" t="n"/>
-      <c r="X28" s="2" t="inlineStr">
-        <is>
-          <t>Any intervention content delivered in the context of a mental health intervention.</t>
-        </is>
-      </c>
+      <c r="X28" s="2" t="n"/>
       <c r="Y28" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -1780,22 +1759,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000250</t>
+          <t>GMHO:0000248</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario</t>
+          <t xml:space="preserve">mental health intervention
+</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A planned process in which a mental health intervention is applied in a given context.</t>
+          <t>An intervention that has the aim of influencing some aspect of mental health.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="E29" s="2" t="n"/>
@@ -1804,41 +1784,30 @@
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. </t>
+          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context, level of engagement and outcomes. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. 
+</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>intervention mechanism of action; participant engagement with intervention; mental health intervention</t>
+          <t>intervention delivery; mental health intervention content</t>
         </is>
       </c>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>mental health intervention scenario plan</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>intervention outcome</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="n"/>
-      <c r="Q29" s="2" t="inlineStr">
-        <is>
-          <t>intervention context</t>
-        </is>
-      </c>
+      <c r="Q29" s="2" t="n"/>
       <c r="R29" s="2" t="n"/>
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="2" t="n"/>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
+      <c r="U29" s="2" t="n"/>
       <c r="V29" s="2" t="n"/>
       <c r="W29" s="2" t="n"/>
       <c r="X29" s="2" t="n"/>
@@ -1853,35 +1822,40 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GMHO:0000260</t>
+          <t>GMHO:0000241</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>mental health intervention scenario plan</t>
+          <t xml:space="preserve">mental health intervention content
+</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>A plan that is realized in a mental health intervention scenario process.</t>
+          <t>An intervention content that is part of a mental health intervention.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>intervention content</t>
         </is>
       </c>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>This class is intended to represent the planned content or delivery of an intervention, whereas the class "mental health intervention scenario" refers to the intervention as it was actually implemented. Distinguishing between these two classes allows for the assessment of intervention fidelity.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>intervention technique</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>intervention dose</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
@@ -1889,16 +1863,16 @@
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
       <c r="R30" s="2" t="n"/>
-      <c r="S30" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:028000</t>
-        </is>
-      </c>
+      <c r="S30" s="2" t="n"/>
       <c r="T30" s="2" t="n"/>
       <c r="U30" s="2" t="n"/>
       <c r="V30" s="2" t="n"/>
       <c r="W30" s="2" t="n"/>
-      <c r="X30" s="2" t="n"/>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>Any intervention content delivered in the context of a mental health intervention.</t>
+        </is>
+      </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -1908,98 +1882,154 @@
       <c r="AA30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>BFO:0000027</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">b is an object aggregate means: b is a material entity consisting exactly of a plurality of objects as member_parts at all times at which b exists. </t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000250</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>A planned process in which a mental health intervention is applied in a given context.</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The "mental health intervention scenario" class captures a "mental health intervention" within a specific context. Mental health interventions (represented as "mental health intervention") could be delivered in different contexts and/or have different outcomes at different times. For example, we could deliver the same intervention ("mental health intervention") two years after its previous delivery or in a different context ("mental health intervention scenario"), and this could lead to different outcomes. </t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>intervention mechanism of action; participant engagement with intervention; mental health intervention</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>intervention outcome</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n"/>
+      <c r="O31" s="2" t="n"/>
+      <c r="P31" s="2" t="n"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="n"/>
+      <c r="S31" s="2" t="n"/>
+      <c r="T31" s="2" t="n"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="n"/>
+      <c r="W31" s="2" t="n"/>
+      <c r="X31" s="2" t="n"/>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="n"/>
+      <c r="AA31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>BCIO:050916</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attendance to intervention sessions, participation in intervention activities, emotionally engaging with intervention content </t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Engagement can involve cognitive, emotional and behavioural engagement with an intervention.</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>The extent to which someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000260</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>mental health intervention scenario plan</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>A plan that is realized in a mental health intervention scenario process.</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>This class is intended to represent the planned content or delivery of an intervention, whereas the class "mental health intervention scenario" refers to the intervention as it was actually implemented. Distinguishing between these two classes allows for the assessment of intervention fidelity.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2" t="n"/>
+      <c r="P32" s="2" t="n"/>
+      <c r="Q32" s="2" t="n"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:028000</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="n"/>
+      <c r="U32" s="2" t="n"/>
+      <c r="V32" s="2" t="n"/>
+      <c r="W32" s="2" t="n"/>
+      <c r="X32" s="2" t="n"/>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="n"/>
+      <c r="AA32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MF:0000016</t>
+          <t>BFO:0000027</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>person</t>
+          <t>object aggregate</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>An extended organism that is a member of the species Homo sapiens.</t>
+          <t xml:space="preserve">b is an object aggregate means: b is a material entity consisting exactly of a plurality of objects as member_parts at all times at which b exists. </t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>extended organism</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>personal history</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -2011,37 +2041,37 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BCIO:015161</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>personal history</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A history that is of a person.</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>history</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>sum of multiple experienced events</t>
+          <t>individual human activity</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attendance to intervention sessions, participation in intervention activities, emotionally engaging with intervention content </t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>A person's history includes the sum of their experiences, which can include experiences relating to their cultural, social and economic context.</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>personal history part</t>
+          <t>Engagement can involve cognitive, emotional and behavioural engagement with an intervention.</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>The extent to which someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -2053,32 +2083,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BCIO:050487</t>
+          <t>MF:0000016</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>personal history part</t>
+          <t>person</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A process that is part of a personal history.</t>
+          <t>An extended organism that is a member of the species Homo sapiens.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>experienced event</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>context of experience</t>
+          <t>extended organism</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>personal history</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -2090,22 +2115,37 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OBI:0000260</t>
+          <t>BCIO:015161</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>personal history</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+          <t>A history that is of a person.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>realizable entity</t>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>sum of multiple experienced events</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>A person's history includes the sum of their experiences, which can include experiences relating to their cultural, social and economic context.</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>personal history part</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -2117,17 +2157,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OBI:0000011</t>
+          <t>BCIO:050487</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>personal history part</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A process that realizes a plan which is the concretization of a plan specification.</t>
+          <t>A process that is part of a personal history.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2135,6 +2175,16 @@
           <t>process</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>experienced event</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>context of experience</t>
+        </is>
+      </c>
       <c r="Y37" t="inlineStr">
         <is>
           <t>External</t>
@@ -2142,222 +2192,191 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>GMHO:0000251</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>population history</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>A history that is of a population.</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>history</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>is an aggregate of personal history; experiences can be captured as 'personal history part'.</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
-      <c r="Q38" s="2" t="n"/>
-      <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="n"/>
-      <c r="T38" s="2" t="n"/>
-      <c r="U38" s="2" t="n"/>
-      <c r="V38" s="2" t="n"/>
-      <c r="W38" s="2" t="n"/>
-      <c r="X38" s="2" t="n"/>
-      <c r="Y38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z38" s="2" t="n"/>
-      <c r="AA38" s="2" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>OBI:0000260</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>plan</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>A plan is a realizable entity that is the inheres in a bearer who is committed to realizing it as a planned process.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>realizable entity</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>OBI:0000011</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>A process that realizes a plan which is the concretization of a plan specification.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>GMHO:0000251</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>population history</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>A history that is of a population.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>is an aggregate of personal history; experiences can be captured as 'personal history part'.</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+      <c r="M40" s="2" t="n"/>
+      <c r="N40" s="2" t="n"/>
+      <c r="O40" s="2" t="n"/>
+      <c r="P40" s="2" t="n"/>
+      <c r="Q40" s="2" t="n"/>
+      <c r="R40" s="2" t="n"/>
+      <c r="S40" s="2" t="n"/>
+      <c r="T40" s="2" t="n"/>
+      <c r="U40" s="2" t="n"/>
+      <c r="V40" s="2" t="n"/>
+      <c r="W40" s="2" t="n"/>
+      <c r="X40" s="2" t="n"/>
+      <c r="Y40" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Z40" s="2" t="n"/>
+      <c r="AA40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>BFO:0000015</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>p is a process = Def. p is an occurrent that has temporal proper parts and for some time t, p s-depends_on some material entity at t. (axiom label in BFO2 Reference: [083-003])</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
+      <c r="Y41" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000005</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">'temporal context of process' OR 'material context of process' </t>
         </is>
       </c>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="N40" s="3" t="n"/>
-      <c r="O40" s="3" t="n"/>
-      <c r="P40" s="3" t="n"/>
-      <c r="Q40" s="3" t="n"/>
-      <c r="R40" s="3" t="n"/>
-      <c r="S40" s="3" t="n"/>
-      <c r="T40" s="3" t="n"/>
-      <c r="U40" s="3" t="n"/>
-      <c r="V40" s="3" t="n"/>
-      <c r="W40" s="3" t="n"/>
-      <c r="X40" s="3" t="n"/>
-      <c r="Y40" s="3" t="inlineStr">
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="n"/>
+      <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
+      <c r="O42" s="3" t="n"/>
+      <c r="P42" s="3" t="n"/>
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="3" t="n"/>
+      <c r="S42" s="3" t="n"/>
+      <c r="T42" s="3" t="n"/>
+      <c r="U42" s="3" t="n"/>
+      <c r="V42" s="3" t="n"/>
+      <c r="W42" s="3" t="n"/>
+      <c r="X42" s="3" t="n"/>
+      <c r="Y42" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="Z40" s="3" t="n"/>
-      <c r="AA40" s="3" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>GMHO:0000268</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>'temporal context of process' OR 'material context of process'</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="n"/>
-      <c r="R41" s="4" t="n"/>
-      <c r="S41" s="4" t="n"/>
-      <c r="T41" s="4" t="n"/>
-      <c r="U41" s="4" t="n"/>
-      <c r="V41" s="4" t="n"/>
-      <c r="W41" s="4" t="n"/>
-      <c r="X41" s="4" t="n"/>
-      <c r="Y41" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="Z41" s="4" t="n"/>
-      <c r="AA41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>SEPIO:0000125</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>research study</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
-      <c r="Y42" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="Z42" s="3" t="n"/>
+      <c r="AA42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2367,24 +2386,32 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>research study</t>
+          <t>process context</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>This class has been replaced by the identical class BCIO:051027 in the Behaviour Change Intervention Ontology (BCIO). Use BCIO:051027 instead.</t>
+        </is>
+      </c>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="n"/>
       <c r="L43" s="3" t="n"/>
@@ -2394,11 +2421,7 @@
       <c r="P43" s="3" t="n"/>
       <c r="Q43" s="3" t="n"/>
       <c r="R43" s="3" t="n"/>
-      <c r="S43" s="3" t="inlineStr">
-        <is>
-          <t>SEPIO:0000125</t>
-        </is>
-      </c>
+      <c r="S43" s="3" t="n"/>
       <c r="T43" s="3" t="n"/>
       <c r="U43" s="3" t="n"/>
       <c r="V43" s="3" t="n"/>
@@ -2415,82 +2438,270 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>BCIO:051027</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SEPIO:0000125</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>research study</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000268</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>research study</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>A planned process that executes some study design or protocol to generate scientific data that is interpreted to test or generate a hypothesis.</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
+      <c r="O46" s="3" t="n"/>
+      <c r="P46" s="3" t="n"/>
+      <c r="Q46" s="3" t="n"/>
+      <c r="R46" s="3" t="n"/>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>SEPIO:0000125</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="n"/>
+      <c r="U46" s="3" t="n"/>
+      <c r="V46" s="3" t="n"/>
+      <c r="W46" s="3" t="n"/>
+      <c r="X46" s="3" t="n"/>
+      <c r="Y46" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z46" s="3" t="n"/>
+      <c r="AA46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>BFO:0000023</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>A realizable entity the manifestation of which brings about some result or end that is not essential to a continuant in virtue of the kind of thing that it is but that can be served or participated in by that kind of continuant in some kinds of natural, social or institutional contexts.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="Y44" t="inlineStr">
+      <c r="Y47" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000006</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>temporal context of process</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">An occurrent that is not dependent on a process but may influence the effect of the process on its outcome. </t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="n"/>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="n"/>
-      <c r="Q45" s="2" t="n"/>
-      <c r="R45" s="2" t="n"/>
-      <c r="S45" s="2" t="n"/>
-      <c r="T45" s="2" t="n"/>
-      <c r="U45" s="2" t="n"/>
-      <c r="V45" s="2" t="n"/>
-      <c r="W45" s="2" t="n"/>
-      <c r="X45" s="2" t="n"/>
-      <c r="Y45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Z45" s="2" t="n"/>
-      <c r="AA45" s="2" t="n"/>
+      <c r="E48" s="3" t="n"/>
+      <c r="F48" s="3" t="n"/>
+      <c r="G48" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>This entity includes time periods, events, etc. 
+This class has been replaced by the identical class BCIO:051028 in the Behaviour Change Intervention Ontology (BCIO). Use BCIO:051028 instead.</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="n"/>
+      <c r="K48" s="3" t="n"/>
+      <c r="L48" s="3" t="n"/>
+      <c r="M48" s="3" t="n"/>
+      <c r="N48" s="3" t="n"/>
+      <c r="O48" s="3" t="n"/>
+      <c r="P48" s="3" t="n"/>
+      <c r="Q48" s="3" t="n"/>
+      <c r="R48" s="3" t="n"/>
+      <c r="S48" s="3" t="n"/>
+      <c r="T48" s="3" t="n"/>
+      <c r="U48" s="3" t="n"/>
+      <c r="V48" s="3" t="n"/>
+      <c r="W48" s="3" t="n"/>
+      <c r="X48" s="3" t="n"/>
+      <c r="Y48" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Z48" s="3" t="n"/>
+      <c r="AA48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BCIO:051028</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An occurrent that is not dependent on a process but may influence the effect of the process on its outcome. </t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>